<commit_message>
resolve merge Corg data conflicts
</commit_message>
<xml_diff>
--- a/Initial data/2025/GeoData.xlsx
+++ b/Initial data/2025/GeoData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1522,471 +1522,473 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ADOM-SL4-10</t>
+          <t>ADOM-SL5-5</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>51.490679</v>
+        <v>51.489518</v>
       </c>
       <c r="C58" t="n">
-        <v>104.236443</v>
+        <v>104.223341</v>
       </c>
       <c r="D58" t="n">
-        <v>9.68</v>
-      </c>
-      <c r="E58" t="inlineStr"/>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E58" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ADOM-SL5-5</t>
+          <t>ADOM-SL5-6</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>51.489518</v>
+        <v>51.489211</v>
       </c>
       <c r="C59" t="n">
-        <v>104.223341</v>
+        <v>104.223398</v>
       </c>
       <c r="D59" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="E59" t="n">
-        <v>80</v>
+        <v>126</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ADOM-SL5-6</t>
+          <t>ADOM-SL5-7</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>51.489211</v>
+        <v>51.488916</v>
       </c>
       <c r="C60" t="n">
-        <v>104.223398</v>
+        <v>104.224301</v>
       </c>
       <c r="D60" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="E60" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ADOM-SL5-7</t>
+          <t>ADOM-SL5-8</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>51.488916</v>
+        <v>51.488792</v>
       </c>
       <c r="C61" t="n">
-        <v>104.224301</v>
+        <v>104.225476</v>
       </c>
       <c r="D61" t="n">
-        <v>7.8</v>
+        <v>8.15</v>
       </c>
       <c r="E61" t="n">
-        <v>118</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ADOM-SL5-8</t>
+          <t>ADOM-SL5-9</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>51.488792</v>
+        <v>51.488542</v>
       </c>
       <c r="C62" t="n">
-        <v>104.225476</v>
+        <v>104.226774</v>
       </c>
       <c r="D62" t="n">
-        <v>8.15</v>
+        <v>7.67</v>
       </c>
       <c r="E62" t="n">
-        <v>108</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ADOM-SL5-9</t>
+          <t>ADOM-SL5-10</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>51.488542</v>
+        <v>51.488464</v>
       </c>
       <c r="C63" t="n">
-        <v>104.226774</v>
+        <v>104.228318</v>
       </c>
       <c r="D63" t="n">
-        <v>7.67</v>
+        <v>7.58</v>
       </c>
       <c r="E63" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ADOM-SL5-10</t>
+          <t>ADOM-SL6-1</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>51.488464</v>
+        <v>51.487512</v>
       </c>
       <c r="C64" t="n">
-        <v>104.228318</v>
+        <v>104.2358</v>
       </c>
       <c r="D64" t="n">
-        <v>7.58</v>
+        <v>7.54</v>
       </c>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>158</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ADOM-SL6-1</t>
+          <t>ADOM-SL6-2</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>51.487512</v>
+        <v>51.487938</v>
       </c>
       <c r="C65" t="n">
-        <v>104.2358</v>
+        <v>104.232506</v>
       </c>
       <c r="D65" t="n">
-        <v>7.54</v>
+        <v>6.61</v>
       </c>
       <c r="E65" t="n">
-        <v>158</v>
+        <v>45</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ADOM-SL6-2</t>
+          <t>ADOM-SL6-3</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>51.487938</v>
+        <v>51.488131</v>
       </c>
       <c r="C66" t="n">
-        <v>104.232506</v>
+        <v>104.229167</v>
       </c>
       <c r="D66" t="n">
-        <v>6.61</v>
+        <v>6.91</v>
       </c>
       <c r="E66" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ADOM-SL6-3</t>
+          <t>ADOM-SL6-4</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>51.488131</v>
+        <v>51.488272</v>
       </c>
       <c r="C67" t="n">
-        <v>104.229167</v>
+        <v>104.225533</v>
       </c>
       <c r="D67" t="n">
-        <v>6.91</v>
+        <v>6.63</v>
       </c>
       <c r="E67" t="n">
-        <v>25</v>
+        <v>-46</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ADOM-SL6-4</t>
+          <t>ADOM-SL6-5</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>51.488272</v>
+        <v>51.488594</v>
       </c>
       <c r="C68" t="n">
-        <v>104.225533</v>
+        <v>104.223923</v>
       </c>
       <c r="D68" t="n">
-        <v>6.63</v>
+        <v>6.7</v>
       </c>
       <c r="E68" t="n">
-        <v>-46</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ADOM-SL6-5</t>
+          <t>ADOM-SL6-6</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>51.488594</v>
+        <v>51.488046</v>
       </c>
       <c r="C69" t="n">
-        <v>104.223923</v>
+        <v>104.225176</v>
       </c>
       <c r="D69" t="n">
-        <v>6.7</v>
+        <v>6.99</v>
       </c>
       <c r="E69" t="n">
-        <v>-2</v>
+        <v>-43</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ADOM-SL6-6</t>
+          <t>ADOM-SL6-7</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>51.488046</v>
+        <v>51.487494</v>
       </c>
       <c r="C70" t="n">
-        <v>104.225176</v>
+        <v>104.228128</v>
       </c>
       <c r="D70" t="n">
-        <v>6.99</v>
+        <v>7.15</v>
       </c>
       <c r="E70" t="n">
-        <v>-43</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ADOM-SL6-7</t>
+          <t>ADOM-SL6-8</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>51.487494</v>
+        <v>51.487368</v>
       </c>
       <c r="C71" t="n">
-        <v>104.228128</v>
+        <v>104.230911</v>
       </c>
       <c r="D71" t="n">
-        <v>7.15</v>
+        <v>6.98</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>-93</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ADOM-SL6-8</t>
+          <t>ADOM-SL6-9</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>51.487368</v>
+        <v>51.487056</v>
       </c>
       <c r="C72" t="n">
-        <v>104.230911</v>
+        <v>104.233501</v>
       </c>
       <c r="D72" t="n">
-        <v>6.98</v>
+        <v>8.01</v>
       </c>
       <c r="E72" t="n">
-        <v>-93</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ADOM-SL6-9</t>
+          <t>ADOM-SL6-10</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>51.487056</v>
+        <v>51.486891</v>
       </c>
       <c r="C73" t="n">
-        <v>104.233501</v>
+        <v>104.235582</v>
       </c>
       <c r="D73" t="n">
-        <v>8.01</v>
+        <v>7.68</v>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ADOM-SL6-10</t>
+          <t>ADOM-SL7-1</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>51.486891</v>
+        <v>51.486065</v>
       </c>
       <c r="C74" t="n">
-        <v>104.235582</v>
+        <v>104.235193</v>
       </c>
       <c r="D74" t="n">
-        <v>7.68</v>
+        <v>7.06</v>
       </c>
       <c r="E74" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ADOM-SL7-1</t>
+          <t>ADOM-SL7-2</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>51.486065</v>
+        <v>51.486513</v>
       </c>
       <c r="C75" t="n">
-        <v>104.235193</v>
+        <v>104.232333</v>
       </c>
       <c r="D75" t="n">
-        <v>7.06</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E75" t="n">
-        <v>52</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ADOM-SL7-2</t>
+          <t>ADOM-SL7-3</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>51.486513</v>
+        <v>51.486908</v>
       </c>
       <c r="C76" t="n">
-        <v>104.232333</v>
+        <v>104.229486</v>
       </c>
       <c r="D76" t="n">
-        <v>8.800000000000001</v>
+        <v>6.9</v>
       </c>
       <c r="E76" t="n">
-        <v>-4</v>
+        <v>-165</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADOM-SL7-3</t>
+          <t>ADOM-SL7-4</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>51.486908</v>
+        <v>51.487308</v>
       </c>
       <c r="C77" t="n">
-        <v>104.229486</v>
+        <v>104.226073</v>
       </c>
       <c r="D77" t="n">
-        <v>6.9</v>
+        <v>8.6</v>
       </c>
       <c r="E77" t="n">
-        <v>-165</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ADOM-SL7-4</t>
+          <t>ADOM-SL7-5</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>51.487308</v>
+        <v>51.487786</v>
       </c>
       <c r="C78" t="n">
-        <v>104.226073</v>
+        <v>104.223797</v>
       </c>
       <c r="D78" t="n">
-        <v>8.6</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="E78" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ADOM-SL7-5</t>
+          <t>ADOM-SL7-6</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>51.487786</v>
+        <v>51.487279</v>
       </c>
       <c r="C79" t="n">
-        <v>104.223797</v>
+        <v>104.223712</v>
       </c>
       <c r="D79" t="n">
-        <v>8.210000000000001</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="E79" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ADOM-SL7-6</t>
+          <t>ADOM-SL7-7</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>51.487279</v>
+        <v>51.485818</v>
       </c>
       <c r="C80" t="n">
-        <v>104.223712</v>
+        <v>104.227152</v>
       </c>
       <c r="D80" t="n">
-        <v>8.640000000000001</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="E80" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ADOM-SL7-7</t>
+          <t>ADOM-SL7-8</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>51.485818</v>
+        <v>51.485331</v>
       </c>
       <c r="C81" t="n">
-        <v>104.227152</v>
+        <v>104.230043</v>
       </c>
       <c r="D81" t="n">
-        <v>8.720000000000001</v>
+        <v>8.67</v>
       </c>
       <c r="E81" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ADOM-SL7-8</t>
+          <t>ADOM-SL7-9</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>51.485331</v>
+        <v>51.485671</v>
       </c>
       <c r="C82" t="n">
-        <v>104.230043</v>
+        <v>104.231312</v>
       </c>
       <c r="D82" t="n">
-        <v>8.67</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="E82" t="n">
         <v>80</v>
@@ -1995,17 +1997,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ADOM-SL7-9</t>
+          <t>ADOM-SL7-10</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>51.485671</v>
+        <v>51.485112</v>
       </c>
       <c r="C83" t="n">
-        <v>104.231312</v>
+        <v>104.234958</v>
       </c>
       <c r="D83" t="n">
-        <v>8.890000000000001</v>
+        <v>7.71</v>
       </c>
       <c r="E83" t="n">
         <v>80</v>
@@ -2014,378 +2016,378 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ADOM-SL7-10</t>
+          <t>ADOM-SL8-1</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>51.485112</v>
+        <v>51.494317</v>
       </c>
       <c r="C84" t="n">
-        <v>104.234958</v>
+        <v>104.251028</v>
       </c>
       <c r="D84" t="n">
-        <v>7.71</v>
+        <v>5.46</v>
       </c>
       <c r="E84" t="n">
-        <v>80</v>
+        <v>163</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ADOM-SL8-1</t>
+          <t>ADOM-SL8-2</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>51.494317</v>
+        <v>51.494874</v>
       </c>
       <c r="C85" t="n">
-        <v>104.251028</v>
+        <v>104.249868</v>
       </c>
       <c r="D85" t="n">
-        <v>5.46</v>
+        <v>4.88</v>
       </c>
       <c r="E85" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ADOM-SL8-2</t>
+          <t>ADOM-SL8-3</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>51.494874</v>
+        <v>51.495363</v>
       </c>
       <c r="C86" t="n">
-        <v>104.249868</v>
+        <v>104.248071</v>
       </c>
       <c r="D86" t="n">
-        <v>4.88</v>
+        <v>5.26</v>
       </c>
       <c r="E86" t="n">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ADOM-SL8-3</t>
+          <t>ADOM-SL8-4</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>51.495363</v>
+        <v>51.496136</v>
       </c>
       <c r="C87" t="n">
-        <v>104.248071</v>
+        <v>104.245657</v>
       </c>
       <c r="D87" t="n">
-        <v>5.26</v>
+        <v>4.64</v>
       </c>
       <c r="E87" t="n">
-        <v>170</v>
+        <v>246</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ADOM-SL8-4</t>
+          <t>ADOM-SL8-5</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>51.496136</v>
+        <v>51.496492</v>
       </c>
       <c r="C88" t="n">
-        <v>104.245657</v>
+        <v>104.244174</v>
       </c>
       <c r="D88" t="n">
-        <v>4.64</v>
+        <v>4.79</v>
       </c>
       <c r="E88" t="n">
-        <v>246</v>
+        <v>287</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ADOM-SL8-5</t>
+          <t>ADOM-SL8-6</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>51.496492</v>
+        <v>51.4944</v>
       </c>
       <c r="C89" t="n">
-        <v>104.244174</v>
+        <v>104.243288</v>
       </c>
       <c r="D89" t="n">
-        <v>4.79</v>
+        <v>6.19</v>
       </c>
       <c r="E89" t="n">
-        <v>287</v>
+        <v>-78</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ADOM-SL8-6</t>
+          <t>ADOM-SL8-7</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>51.4944</v>
+        <v>51.494249</v>
       </c>
       <c r="C90" t="n">
-        <v>104.243288</v>
+        <v>104.245225</v>
       </c>
       <c r="D90" t="n">
-        <v>6.19</v>
+        <v>5.17</v>
       </c>
       <c r="E90" t="n">
-        <v>-78</v>
+        <v>174</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ADOM-SL8-7</t>
+          <t>ADOM-SL8-8</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>51.494249</v>
+        <v>51.493909</v>
       </c>
       <c r="C91" t="n">
-        <v>104.245225</v>
+        <v>104.246603</v>
       </c>
       <c r="D91" t="n">
-        <v>5.17</v>
+        <v>8.51</v>
       </c>
       <c r="E91" t="n">
-        <v>174</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ADOM-SL8-8</t>
+          <t>ADOM-SL8-9</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>51.493909</v>
+        <v>51.493895</v>
       </c>
       <c r="C92" t="n">
-        <v>104.246603</v>
+        <v>104.246718</v>
       </c>
       <c r="D92" t="n">
-        <v>8.51</v>
+        <v>4.79</v>
       </c>
       <c r="E92" t="n">
-        <v>-17</v>
+        <v>189</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ADOM-SL8-9</t>
+          <t>ADOM-SL8-10</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>51.493895</v>
+        <v>51.493481</v>
       </c>
       <c r="C93" t="n">
-        <v>104.246718</v>
+        <v>104.250557</v>
       </c>
       <c r="D93" t="n">
-        <v>4.79</v>
+        <v>5.72</v>
       </c>
       <c r="E93" t="n">
-        <v>189</v>
+        <v>59</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ADOM-SL8-10</t>
+          <t>ADOM-SL9-1</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>51.493481</v>
+        <v>51.490657</v>
       </c>
       <c r="C94" t="n">
-        <v>104.250557</v>
+        <v>104.241843</v>
       </c>
       <c r="D94" t="n">
-        <v>5.72</v>
+        <v>5.99</v>
       </c>
       <c r="E94" t="n">
-        <v>59</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ADOM-SL9-1</t>
+          <t>ADOM-SL9-2</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>51.490657</v>
+        <v>51.493049</v>
       </c>
       <c r="C95" t="n">
-        <v>104.241843</v>
+        <v>104.2428</v>
       </c>
       <c r="D95" t="n">
-        <v>5.99</v>
+        <v>7.23</v>
       </c>
       <c r="E95" t="n">
-        <v>20</v>
+        <v>173</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ADOM-SL9-2</t>
+          <t>ADOM-SL9-3</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>51.493049</v>
+        <v>51.490264</v>
       </c>
       <c r="C96" t="n">
-        <v>104.2428</v>
+        <v>104.244545</v>
       </c>
       <c r="D96" t="n">
-        <v>7.23</v>
+        <v>7.1</v>
       </c>
       <c r="E96" t="n">
-        <v>173</v>
+        <v>140</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ADOM-SL9-3</t>
+          <t>ADOM-SL9-4</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>51.490264</v>
+        <v>51.490211</v>
       </c>
       <c r="C97" t="n">
-        <v>104.244545</v>
+        <v>104.245922</v>
       </c>
       <c r="D97" t="n">
-        <v>7.1</v>
+        <v>6.98</v>
       </c>
       <c r="E97" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ADOM-SL9-4</t>
+          <t>ADOM-SL9-5</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>51.490211</v>
+        <v>51.490264</v>
       </c>
       <c r="C98" t="n">
-        <v>104.245922</v>
+        <v>104.247637</v>
       </c>
       <c r="D98" t="n">
-        <v>6.98</v>
+        <v>7.02</v>
       </c>
       <c r="E98" t="n">
-        <v>143</v>
+        <v>110</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ADOM-SL9-5</t>
+          <t>ADOM-SL9-6</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>51.490264</v>
+        <v>51.49063</v>
       </c>
       <c r="C99" t="n">
-        <v>104.247637</v>
+        <v>104.249402</v>
       </c>
       <c r="D99" t="n">
-        <v>7.02</v>
+        <v>7.4</v>
       </c>
       <c r="E99" t="n">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ADOM-SL9-6</t>
+          <t>ADOM-SL9-7</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>51.49063</v>
+        <v>51.491006</v>
       </c>
       <c r="C100" t="n">
-        <v>104.249402</v>
+        <v>104.250919</v>
       </c>
       <c r="D100" t="n">
-        <v>7.4</v>
+        <v>7.11</v>
       </c>
       <c r="E100" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ADOM-SL9-7</t>
+          <t>ADOM-SL9-8</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>51.491006</v>
+        <v>51.491683</v>
       </c>
       <c r="C101" t="n">
-        <v>104.250919</v>
+        <v>104.251002</v>
       </c>
       <c r="D101" t="n">
-        <v>7.11</v>
+        <v>5.6</v>
       </c>
       <c r="E101" t="n">
-        <v>125</v>
+        <v>52</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ADOM-SL9-8</t>
+          <t>ADOM-SL9-9</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>51.491683</v>
+        <v>51.491824</v>
       </c>
       <c r="C102" t="n">
-        <v>104.251002</v>
+        <v>104.250445</v>
       </c>
       <c r="D102" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="E102" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ADOM-SL9-9</t>
+          <t>ADOM-SL9-10</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>51.491824</v>
+        <v>51.492207</v>
       </c>
       <c r="C103" t="n">
-        <v>104.250445</v>
+        <v>104.247648</v>
       </c>
       <c r="D103" t="n">
-        <v>5.9</v>
+        <v>6.56</v>
       </c>
       <c r="E103" t="n">
         <v>42</v>
@@ -2394,36 +2396,36 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ADOM-SL9-10</t>
+          <t>ADOM-SL9-11</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>51.492207</v>
+        <v>51.49234</v>
       </c>
       <c r="C104" t="n">
-        <v>104.247648</v>
+        <v>104.246479</v>
       </c>
       <c r="D104" t="n">
-        <v>6.56</v>
+        <v>6.65</v>
       </c>
       <c r="E104" t="n">
-        <v>42</v>
+        <v>69</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ADOM-SL9-11</t>
+          <t>ADOM-SL9-12</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>51.49234</v>
+        <v>51.492785</v>
       </c>
       <c r="C105" t="n">
-        <v>104.246479</v>
+        <v>104.244319</v>
       </c>
       <c r="D105" t="n">
-        <v>6.65</v>
+        <v>6.79</v>
       </c>
       <c r="E105" t="n">
         <v>69</v>
@@ -2432,17 +2434,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ADOM-SL9-12</t>
+          <t>ADOM-SL9-13</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>51.492785</v>
+        <v>51.492921</v>
       </c>
       <c r="C106" t="n">
-        <v>104.244319</v>
+        <v>104.242403</v>
       </c>
       <c r="D106" t="n">
-        <v>6.79</v>
+        <v>6.1</v>
       </c>
       <c r="E106" t="n">
         <v>69</v>
@@ -2451,112 +2453,112 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ADOM-SL9-13</t>
+          <t>ADOM-SL10-1</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>51.492921</v>
+        <v>51.488401</v>
       </c>
       <c r="C107" t="n">
-        <v>104.242403</v>
+        <v>104.241367</v>
       </c>
       <c r="D107" t="n">
-        <v>6.1</v>
+        <v>4.19</v>
       </c>
       <c r="E107" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ADOM-SL10-1</t>
+          <t>ADOM-SL10-2</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>51.488401</v>
+        <v>51.488007</v>
       </c>
       <c r="C108" t="n">
-        <v>104.241367</v>
+        <v>104.242372</v>
       </c>
       <c r="D108" t="n">
-        <v>4.19</v>
+        <v>4.27</v>
       </c>
       <c r="E108" t="n">
-        <v>25</v>
+        <v>115</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ADOM-SL10-2</t>
+          <t>ADOM-SL10-3</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>51.488007</v>
+        <v>51.487939</v>
       </c>
       <c r="C109" t="n">
-        <v>104.242372</v>
+        <v>104.244479</v>
       </c>
       <c r="D109" t="n">
-        <v>4.27</v>
+        <v>4.01</v>
       </c>
       <c r="E109" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ADOM-SL10-3</t>
+          <t>ADOM-SL10-4</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>51.487939</v>
+        <v>51.488319</v>
       </c>
       <c r="C110" t="n">
-        <v>104.244479</v>
+        <v>104.244186</v>
       </c>
       <c r="D110" t="n">
-        <v>4.01</v>
+        <v>4.54</v>
       </c>
       <c r="E110" t="n">
-        <v>113</v>
+        <v>-83</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ADOM-SL10-4</t>
+          <t>ADOM-SL10-5</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>51.488319</v>
+        <v>51.487859</v>
       </c>
       <c r="C111" t="n">
-        <v>104.244186</v>
+        <v>104.246384</v>
       </c>
       <c r="D111" t="n">
-        <v>4.54</v>
+        <v>5.49</v>
       </c>
       <c r="E111" t="n">
-        <v>-83</v>
+        <v>-110</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ADOM-SL10-5</t>
+          <t>ADOM-SL10-6</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>51.487859</v>
+        <v>51.488817</v>
       </c>
       <c r="C112" t="n">
-        <v>104.246384</v>
+        <v>104.24684</v>
       </c>
       <c r="D112" t="n">
-        <v>5.49</v>
+        <v>4.87</v>
       </c>
       <c r="E112" t="n">
         <v>-110</v>
@@ -2565,95 +2567,76 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ADOM-SL10-6</t>
+          <t>ADOM-SL10-7</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>51.488817</v>
+        <v>51.489152</v>
       </c>
       <c r="C113" t="n">
-        <v>104.24684</v>
+        <v>104.24603</v>
       </c>
       <c r="D113" t="n">
-        <v>4.87</v>
+        <v>5.47</v>
       </c>
       <c r="E113" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ADOM-SL10-7</t>
+          <t>ADOM-SL10-8</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>51.489152</v>
+        <v>51.489235</v>
       </c>
       <c r="C114" t="n">
-        <v>104.24603</v>
+        <v>104.244566</v>
       </c>
       <c r="D114" t="n">
-        <v>5.47</v>
+        <v>4.82</v>
       </c>
       <c r="E114" t="n">
-        <v>-105</v>
+        <v>-88</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ADOM-SL10-8</t>
+          <t>ADOM-SL10-9</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>51.489235</v>
+        <v>51.489188</v>
       </c>
       <c r="C115" t="n">
-        <v>104.244566</v>
+        <v>104.243469</v>
       </c>
       <c r="D115" t="n">
-        <v>4.82</v>
+        <v>4.09</v>
       </c>
       <c r="E115" t="n">
-        <v>-88</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ADOM-SL10-9</t>
+          <t>ADOM-SL10-10</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>51.489188</v>
+        <v>51.489219</v>
       </c>
       <c r="C116" t="n">
-        <v>104.243469</v>
+        <v>104.241603</v>
       </c>
       <c r="D116" t="n">
-        <v>4.09</v>
+        <v>5.59</v>
       </c>
       <c r="E116" t="n">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>ADOM-SL10-10</t>
-        </is>
-      </c>
-      <c r="B117" t="n">
-        <v>51.489219</v>
-      </c>
-      <c r="C117" t="n">
-        <v>104.241603</v>
-      </c>
-      <c r="D117" t="n">
-        <v>5.59</v>
-      </c>
-      <c r="E117" t="n">
         <v>-107</v>
       </c>
     </row>

</xml_diff>